<commit_message>
Fix classifier output encoding
</commit_message>
<xml_diff>
--- a/outputs/issue_classification_summary.xlsx
+++ b/outputs/issue_classification_summary.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Issue Distribution" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Restaurant Issues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="High Confidence Examples" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Low Confidence Examples" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,10 +443,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3254</v>
+        <v>3304</v>
       </c>
       <c r="C2" t="n">
-        <v>52.83</v>
+        <v>53.65</v>
       </c>
     </row>
     <row r="3">
@@ -454,10 +456,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>927</v>
+        <v>938</v>
       </c>
       <c r="C3" t="n">
-        <v>15.05</v>
+        <v>15.23</v>
       </c>
     </row>
     <row r="4">
@@ -467,10 +469,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="C4" t="n">
-        <v>8.52</v>
+        <v>8.460000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -480,10 +482,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="C5" t="n">
-        <v>6.53</v>
+        <v>6.36</v>
       </c>
     </row>
     <row r="6">
@@ -493,10 +495,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>391</v>
+        <v>347</v>
       </c>
       <c r="C6" t="n">
-        <v>6.35</v>
+        <v>5.63</v>
       </c>
     </row>
     <row r="7">
@@ -506,10 +508,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C7" t="n">
-        <v>4.12</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="8">
@@ -519,10 +521,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C8" t="n">
-        <v>3.65</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="9">
@@ -532,10 +534,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C9" t="n">
-        <v>1.49</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="10">
@@ -545,10 +547,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C10" t="n">
-        <v>1.06</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="11">
@@ -558,10 +560,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
     </row>
   </sheetData>
@@ -642,34 +644,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" t="n">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="F2" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H2" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="I2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J2" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="K2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -688,22 +690,22 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F3" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G3" t="n">
         <v>11</v>
       </c>
       <c r="H3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I3" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J3" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K3" t="n">
         <v>8</v>
@@ -716,31 +718,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E4" t="n">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="F4" t="n">
         <v>39</v>
       </c>
       <c r="G4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H4" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J4" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="K4" t="n">
         <v>10</v>
@@ -753,34 +755,34 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E5" t="n">
-        <v>842</v>
+        <v>853</v>
       </c>
       <c r="F5" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H5" t="n">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="I5" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="J5" t="n">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="K5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -790,7 +792,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
         <v>3</v>
@@ -799,25 +801,25 @@
         <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>455</v>
+        <v>468</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H6" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J6" t="n">
         <v>99</v>
       </c>
       <c r="K6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -827,34 +829,906 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E7" t="n">
-        <v>818</v>
+        <v>834</v>
       </c>
       <c r="F7" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G7" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H7" t="n">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="I7" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J7" t="n">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="K7" t="n">
-        <v>26</v>
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>review_text</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>predicted_issue_category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>adyar ananda bhavan in gandhipuram is offering authentic vegetarian south indian classics, north indian, and tandoori delights, along with indo-chinese combos. all the items are delicious with great taste and servvd hot. …</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.968511489774012</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>i liked food here, we ordered fried rice, gobi manchurian watermelon juice and in desserts jamun and rasmalai, it was good.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Service Quality</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8259535515831755</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>the place is not at all maintained…there is a broken glass that hasn’t been replaced and an overflowing trash can that hasn’t been attended to. you also cannot tip the employees and the food quantity is very very less like for a ₹90 pongal you get a small cup of portion….the panned butter masala is extremely sweet…dissapointed.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9906571714505228</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mr.saravana served me kothu parotta, which i tried first in my life and it was awsm…</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Service Quality</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9456137615927044</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gobi manchurian poor quality chef dont know what it is, too much sauce and salt and preservatives, too noisy atmosphere, same glove worn by waiters infact they touch lot of places and food too with glove, bare hand allows them …</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8641858723449644</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>the quantity of pongal was very less. for the mini tiffin- 165rs, the coffee was not provided. the quantity and quality of breakfast has become 😞 bad and not worth for money. …</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.9931314275994005</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>food is sour , not worth money 135 dosa full sour taste , idly was better . not visiting again</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Service Quality</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.914421192961391</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>the food is good. they serve everything hot and fresh. we sat at table 16 the waiter assigned ms amruta varshini was very swift with her service and asked us about our specifications, didn't make us wait too long.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.990048493058316</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>the meals taste very good. i ordered through swiggy and the price was around ₹150, which is totally worth it. you must try the mushroom biryani as well. for takeaway orders, it takes some time to prepare, so be ready to wait.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9942092543773607</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>"the dosa served to me appeared to be made from overly sour batter. the taste and smell were unpleasant, and i was unable to finish the meal. i was disappointed with the food quality and hope the restaurant pays more attention to freshness and quality control."</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.96516495695352</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t># a2b gandhipuram: a disappointing decline once a culinary highlight in gandhipuram, a2b has sadly fallen from grace. the …</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.9909155535744804</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>food and ambience was good. fully ac dining area. washroom and toilet was outside. …</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ambience &amp; Seating</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.9334839374187746</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>good atmosphere and quality food.the other main highlight of this outlet is its opens on 6:30 am, where you can’t find any other vegetarian option in this locality.neat and clean premises.congested wash area is the only negative find there.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.9917796459386161</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>i visited the adyar ananda bhavan outlet in gandhipuram last night.the quantity and quality of the food were reasonably good, but the prices were on the higher side. however, the service style and the staff's demeanor were somewhat …</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.9562674353827143</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>worst experience i've had at an a2b, especially in coimbatore gandhipuram branch. the food quality was far below expectations. the sambar tasted bland and felt …</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.9834647754321362</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>it was an unplanned quick visit during our ride to kovai. just checked in to have some cool drinks, and the order process was tiring, and nobody was there to help with. got the order delivered only after 15 minutes that, too, just 2 orange …</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.9890470461084387</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>we visited hotel and had to wait for a very long time. the servers were extremely slow and the service was delayed. this should not happen, especially for a place with such a good reputation. please ensure your staff attend to customers more quickly and efficiently.”</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.8455855013213509</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>today during dinner, the service quality was very disappointing. none of the staff seemed attentive to customers. the waiters and captains were moving around without any focus, and there was no proper monitoring of the floor. …</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.9714525232118988</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>i have been visiting this place once in a while since 9 years. i just noticed that i never reviewed this place yet. the food here is exceptionally good usually though there was a small difference today. i would have reduced more stars for …</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Food Quantity &amp; Value for Money</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.8193446783622443</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>i normally eat in a2b but this one the staff were not good. they were slow and made me wait a lot. i've given 4 starts for food.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cleanliness &amp; Restroom Hygiene</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.9616236398005631</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>review_text</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>predicted_issue_category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>i had a sweet paniyaram which is very good taste but outer surface is very hard to bite which made my teeth painful. please make that as soft as possible to enjoy the delicious</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.4221703169572218</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>a2b used to maintain their brand name, food quality and taste in all their branches... here also they maintaining the same. this hotel has vast area for dine in. . quick responded services are available here. . . need not to spend more than …</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Food Variety &amp; Fast Service</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.4222583553955247</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sakthivel received us well and had good lunch here.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Slow Service &amp; Staff Negligence</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.4954885052329822</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>provided stale food during lunch. pls dont visit a2b for lunch. they dont respect customer and their feedback.waste of money and stomach will spoil because of their food. differently not value for money. all gravy will be watery and will …</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Slow Service &amp; Staff Negligence</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.4963405763389222</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>i’ve visited this outlet multiple times in 2023-2024, indeed it’s a good place for breakfast. they’ve got lots of varieties in dosa and many other south indian dishes. it’s usually full in the morning and you might have to wait some time to …</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.451860181516931</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>horrible food experience i had there ,,, they served me very stale idly and told me if they put hot sambar idly becomes hot,,, i changed idly to upma,,they served stale upma and it was yuk,,, i really appreciate a2b serving people ,,but few …</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Food Variety &amp; Fast Service</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2843351633863573</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>it's pure vegetarian restaurant. all kind of item you would get. starting with breakfast pongal, rawa khichadi (upma), etc. veriety of dosa, every day there is one special dosa.. today it was paneer dosa... you also get dumplings , mini …</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Service Quality</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.4850277232496833</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>worst service got in lunch. i visited more than 40 a2bs around tamilnadu but this was very poor service. all servers are from other state and they don't know and understand tamil which cause so many chaos for my elders.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Service Quality</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.3510511496918333</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ordered poori and dosa from swiggy today. poori was dry and too oily. found a worm in chutney. i called to restaurant to inform this they didn’t answer me and hanged call.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.2602415752905459</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>worst ever service don't choose a2b shastri road better prefer shri sangeethas restaurant for quick dine service …</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Slow Service &amp; Staff Negligence</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.4680836175257094</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>we stepped in during late hours for dinner. durga waited on us with a great smile. she managed to get all of the orders without making us wait for a longer time. i would definitely visit back especially to meet her again 🤪 …</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Slow Service &amp; Staff Negligence</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.4883630107730401</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>"i am writing to express my disappointment regarding the service at your restaurant during my recent visit. we waited for more than half an hour after being seated, but no staff member came to take our food order, even though we tried to …</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Slow Service &amp; Staff Negligence</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.331219954272798</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>worst experience, around 30 mins, nobody came to table, they turned face other side. they never bother about customer. came out without having food, around 30 mins</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.4789770611466073</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>worst a2b restaurant i have ever seen no proper service persons . taking too long time to serve food . it should be closed or else change the manger or supervisor to take care</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.4712951563330148</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>whatever you order its not there. dosa not there, manchurian not there …</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.4914573385456499</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>very bad experience. it took 15 mins for someone to take the order. very few people are available for service. hardly any items are available, which is very surprising on a long weekend sunday. strictly not advisable for people planning to have a quick bite before boarding train.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.4343627224523933</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Geetham</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>if you are looking for for south indian authentic vegetarian food. this is the place for you . don’t miss to taste paayasam that’s been served with every thali. quick service with happy meal</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.4717969110226677</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Geetham</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>quality of food degraded over the years. traditional tamilnadu meals quality is no more available in this resturant. high content of oil in every dish makes it unhealthy to eat at this place. resturant management should concentrate of food quality. service and atmosphere is decent and fast.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.4224800924759259</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Geetham</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>nice ambience , clean restrooms , lovely food.. i love how they maintain their standards with consistency with respect to food.. loved their pista rose kunafa totally.. everything was delivered without delay, nice service.. overall a great experience! ♥️💐 …</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Slow Service &amp; Staff Negligence</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.4125097033794984</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Geetham</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>restaurant is very good, comforting and have very nice ambience. food is very good, all vegetarian menu and tastes very good. staff is also very nice, quite friendly and also able to understand hindi. menu is very vast including chinese, …</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Food Variety &amp; Fast Service</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.4940951555090529</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run review pipeline on raw_reviews_new
</commit_message>
<xml_diff>
--- a/outputs/issue_classification_summary.xlsx
+++ b/outputs/issue_classification_summary.xlsx
@@ -443,10 +443,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3304</v>
+        <v>3018</v>
       </c>
       <c r="C2" t="n">
-        <v>53.65</v>
+        <v>53.17</v>
       </c>
     </row>
     <row r="3">
@@ -456,10 +456,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>938</v>
+        <v>849</v>
       </c>
       <c r="C3" t="n">
-        <v>15.23</v>
+        <v>14.96</v>
       </c>
     </row>
     <row r="4">
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>521</v>
+        <v>458</v>
       </c>
       <c r="C4" t="n">
-        <v>8.460000000000001</v>
+        <v>8.07</v>
       </c>
     </row>
     <row r="5">
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>392</v>
+        <v>378</v>
       </c>
       <c r="C5" t="n">
-        <v>6.36</v>
+        <v>6.66</v>
       </c>
     </row>
     <row r="6">
@@ -495,10 +495,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="C6" t="n">
-        <v>5.63</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="7">
@@ -508,10 +508,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C7" t="n">
-        <v>4.06</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="8">
@@ -521,10 +521,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
-        <v>3.73</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="9">
@@ -534,10 +534,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C9" t="n">
-        <v>1.41</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="10">
@@ -547,10 +547,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C10" t="n">
-        <v>1.09</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="11">
@@ -560,10 +560,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C11" t="n">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
     </row>
   </sheetData>
@@ -644,34 +644,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E2" t="n">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="G2" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="I2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J2" t="n">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="K2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -681,34 +681,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>209</v>
+        <v>156</v>
       </c>
       <c r="F3" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="G3" t="n">
         <v>11</v>
       </c>
       <c r="H3" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I3" t="n">
+        <v>24</v>
+      </c>
+      <c r="J3" t="n">
         <v>36</v>
       </c>
-      <c r="J3" t="n">
-        <v>68</v>
-      </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -718,34 +718,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E4" t="n">
-        <v>373</v>
+        <v>342</v>
       </c>
       <c r="F4" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H4" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I4" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="J4" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="K4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -755,34 +755,34 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E5" t="n">
-        <v>853</v>
+        <v>825</v>
       </c>
       <c r="F5" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H5" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="I5" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="J5" t="n">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="K5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -792,31 +792,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>468</v>
+        <v>359</v>
       </c>
       <c r="F6" t="n">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="G6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H6" t="n">
         <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J6" t="n">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="K6" t="n">
         <v>6</v>
@@ -829,31 +829,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E7" t="n">
-        <v>834</v>
+        <v>771</v>
       </c>
       <c r="F7" t="n">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="G7" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H7" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I7" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J7" t="n">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="K7" t="n">
         <v>24</v>
@@ -903,7 +903,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>adyar ananda bhavan in gandhipuram is offering authentic vegetarian south indian classics, north indian, and tandoori delights, along with indo-chinese combos. all the items are delicious with great taste and servvd hot. …</t>
+          <t>the quantity of pongal was very less. for the mini tiffin- 165rs, the coffee was not provided. the quantity and quality of breakfast has become 😞 bad and not worth for money. …</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.968511489774012</v>
+        <v>0.8933333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -923,16 +923,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>i liked food here, we ordered fried rice, gobi manchurian watermelon juice and in desserts jamun and rasmalai, it was good.</t>
+          <t>too expensive and not worth the money at all . i would suggest to avoid any chaats here .</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Service Quality</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8259535515831755</v>
+        <v>0.8366666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -943,16 +943,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>the place is not at all maintained…there is a broken glass that hasn’t been replaced and an overflowing trash can that hasn’t been attended to. you also cannot tip the employees and the food quantity is very very less like for a ₹90 pongal you get a small cup of portion….the panned butter masala is extremely sweet…dissapointed.</t>
+          <t>located near megastar theater... parking available... taste is good... …</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Food Quantity &amp; Value for Money</t>
+          <t>Parking &amp; Accessibility</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.9906571714505228</v>
+        <v>0.8366666666666667</v>
       </c>
     </row>
     <row r="5">
@@ -963,87 +963,87 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>mr.saravana served me kothu parotta, which i tried first in my life and it was awsm…</t>
+          <t>yesterday i had my breakfast where the service was too late because where there was no cooperation among the workers where they are fighting for the ordered plate due theor fight the foods are provided too late and main thing i observed the …</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Service Quality</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.9456137615927044</v>
+        <v>0.8433333333333334</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>gobi manchurian poor quality chef dont know what it is, too much sauce and salt and preservatives, too noisy atmosphere, same glove worn by waiters infact they touch lot of places and food too with glove, bare hand allows them …</t>
+          <t>the food quality is great and taste is very good.the price is little high but its worth for the taste and quantity well we have ordered a panner briyani, the amount of panner is very high. …</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.8641858723449644</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>the quantity of pongal was very less. for the mini tiffin- 165rs, the coffee was not provided. the quantity and quality of breakfast has become 😞 bad and not worth for money. …</t>
+          <t>ambience was neat and clean. seating was so comfortable and cozy extraordinary service and friendly staffs. …</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Food Quantity &amp; Value for Money</t>
+          <t>Ambience &amp; Seating</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.9931314275994005</v>
+        <v>0.8433333333333334</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>food is sour , not worth money 135 dosa full sour taste , idly was better . not visiting again</t>
+          <t>high class vegetrian restaurant near to chatram bus stand at trichy. karur road#karurbypass junction near. parking available. quality ok</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Service Quality</t>
+          <t>Parking &amp; Accessibility</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.914421192961391</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>the food is good. they serve everything hot and fresh. we sat at table 16 the waiter assigned ms amruta varshini was very swift with her service and asked us about our specifications, didn't make us wait too long.</t>
+          <t>i went after seeing ratings. it is complete use less. not worth the money. i ordered nattu kozhi man satti fry. they costed 320 they gave only 2 of pieces. don’t trust the ratings. it seems they pay to social media influencers to promote their shop.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1052,18 +1052,18 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.990048493058316</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>the meals taste very good. i ordered through swiggy and the price was around ₹150, which is totally worth it. you must try the mushroom biryani as well. for takeaway orders, it takes some time to prepare, so be ready to wait.</t>
+          <t>chicken was full of skin and no flesh not worthy for the price</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1072,18 +1072,18 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.9942092543773607</v>
+        <v>0.8266666666666667</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>"the dosa served to me appeared to be made from overly sour batter. the taste and smell were unpleasant, and i was unable to finish the meal. i was disappointed with the food quality and hope the restaurant pays more attention to freshness and quality control."</t>
+          <t>simply overrated. briyani - not that great, doesn't justify it's price. nv meals priced closer to rs.400, but not worth the spend.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1092,58 +1092,58 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.96516495695352</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sangeetha</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t># a2b gandhipuram: a disappointing decline once a culinary highlight in gandhipuram, a2b has sadly fallen from grace. the …</t>
+          <t>neat and clean. it is fit to certain class of people. no car parking available. indoor and outdoor units are there. sincerity is seen in every dishes prepared and tasty. but for heaven shake, don't go for their parcel service. worst of …</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Food Quantity &amp; Value for Money</t>
+          <t>Parking &amp; Accessibility</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.9909155535744804</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Saravana Bhavan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>food and ambience was good. fully ac dining area. washroom and toilet was outside. …</t>
+          <t>worst cleanliness. prices are too high and the food is not worth the taste. the only item i would recommend is mushroom biryani; apart from that, nothing tastes good. …</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ambience &amp; Seating</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.9334839374187746</v>
+        <v>0.8233333333333334</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sree Annapoorna</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>good atmosphere and quality food.the other main highlight of this outlet is its opens on 6:30 am, where you can’t find any other vegetarian option in this locality.neat and clean premises.congested wash area is the only negative find there.</t>
+          <t>my life la one of the biggest mistake i purchased this hotel food per meals 180rs toooo expensive and tooo bad and not worth this price better option buy 50rs meal vandikadai</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1152,18 +1152,18 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.9917796459386161</v>
+        <v>0.8133333333333334</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sree Annapoorna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>i visited the adyar ananda bhavan outlet in gandhipuram last night.the quantity and quality of the food were reasonably good, but the prices were on the higher side. however, the service style and the staff's demeanor were somewhat …</t>
+          <t>food: the taste is average. not worth the hype. i've had breakfast,lunch,dinner here. talking about the breakfast: …</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1172,18 +1172,18 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.9562674353827143</v>
+        <v>0.8533333333333334</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sree Annapoorna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>worst experience i've had at an a2b, especially in coimbatore gandhipuram branch. the food quality was far below expectations. the sambar tasted bland and felt …</t>
+          <t>went for dinner with family, had the best filter coffee and ghee podi dosa here. not too costly, and the service was good. would come again for the coffee soon 😁 …</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1192,38 +1192,38 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.9834647754321362</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sree Annapoorna</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>it was an unplanned quick visit during our ride to kovai. just checked in to have some cool drinks, and the order process was tiring, and nobody was there to help with. got the order delivered only after 15 minutes that, too, just 2 orange …</t>
+          <t>good veg restaurant at lakshmi complex , parking available here - paid.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Food Quantity &amp; Value for Money</t>
+          <t>Parking &amp; Accessibility</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.9890470461084387</v>
+        <v>0.8366666666666667</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sree Annapoorna</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>we visited hotel and had to wait for a very long time. the servers were extremely slow and the service was delayed. this should not happen, especially for a place with such a good reputation. please ensure your staff attend to customers more quickly and efficiently.”</t>
+          <t>pongal is half the quantity for the price vadai is very small size coffee not taste and not heat</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1232,18 +1232,18 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.8455855013213509</v>
+        <v>0.8033333333333333</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Sree Annapoorna</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>today during dinner, the service quality was very disappointing. none of the staff seemed attentive to customers. the waiters and captains were moving around without any focus, and there was no proper monitoring of the floor. …</t>
+          <t>excellent quality. worth much for the price</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1252,18 +1252,18 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.9714525232118988</v>
+        <v>0.8266666666666667</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Namma Veedu Vasanta Bhavan</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>i have been visiting this place once in a while since 9 years. i just noticed that i never reviewed this place yet. the food here is exceptionally good usually though there was a small difference today. i would have reduced more stars for …</t>
+          <t>food was just average for the price . so much waiting time and not worth the ambience and hype the restaurant had</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1272,27 +1272,27 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.8193446783622443</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>A2B</t>
+          <t>Namma Veedu Vasanta Bhavan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>i normally eat in a2b but this one the staff were not good. they were slow and made me wait a lot. i've given 4 starts for food.</t>
+          <t>what a terrible experience and definitely not worth the money paid. i understand every new establishment has teething issues, this one is just with the attitude. …</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cleanliness &amp; Restroom Hygiene</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.9616236398005631</v>
+        <v>0.83</v>
       </c>
     </row>
   </sheetData>
@@ -1339,16 +1339,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>i had a sweet paniyaram which is very good taste but outer surface is very hard to bite which made my teeth painful. please make that as soft as possible to enjoy the delicious</t>
+          <t>i liked food here, we ordered fried rice, gobi manchurian watermelon juice and in desserts jamun and rasmalai, it was good.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Service Quality</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.4221703169572218</v>
+        <v>0.3866666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -1359,16 +1359,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>a2b used to maintain their brand name, food quality and taste in all their branches... here also they maintaining the same. this hotel has vast area for dine in. . quick responded services are available here. . . need not to spend more than …</t>
+          <t>mr.saravana served me kothu parotta, which i tried first in my life and it was awsm…</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Food Variety &amp; Fast Service</t>
+          <t>Service Quality</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.4222583553955247</v>
+        <v>0.4066666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -1379,16 +1379,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sakthivel received us well and had good lunch here.</t>
+          <t>gobi manchurian poor quality chef dont know what it is, too much sauce and salt and preservatives, too noisy atmosphere, same glove worn by waiters infact they touch lot of places and food too with glove, bare hand allows them …</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Slow Service &amp; Staff Negligence</t>
+          <t>Poor Experience &amp; Food Hygiene Complaints</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.4954885052329822</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="5">
@@ -1399,16 +1399,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>provided stale food during lunch. pls dont visit a2b for lunch. they dont respect customer and their feedback.waste of money and stomach will spoil because of their food. differently not value for money. all gravy will be watery and will …</t>
+          <t>wonderful menu and freshness of food 🥘 my son enjoyed eating their homemade sweet kolukattai …</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Slow Service &amp; Staff Negligence</t>
+          <t>Food Variety &amp; Fast Service</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.4963405763389222</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6">
@@ -1419,16 +1419,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>i’ve visited this outlet multiple times in 2023-2024, indeed it’s a good place for breakfast. they’ve got lots of varieties in dosa and many other south indian dishes. it’s usually full in the morning and you might have to wait some time to …</t>
+          <t>if you want to eat pure veg in tamilnadu then this place is for you. very supportive staff and most importantly very fast service they provide. and food is also very delicious... must try this place.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Slow Service &amp; Staff Negligence</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.451860181516931</v>
+        <v>0.3466666666666667</v>
       </c>
     </row>
     <row r="7">
@@ -1439,16 +1439,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>horrible food experience i had there ,,, they served me very stale idly and told me if they put hot sambar idly becomes hot,,, i changed idly to upma,,they served stale upma and it was yuk,,, i really appreciate a2b serving people ,,but few …</t>
+          <t>food is sour , not worth money 135 dosa full sour taste , idly was better . not visiting again</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Food Variety &amp; Fast Service</t>
+          <t>Service Quality</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.2843351633863573</v>
+        <v>0.2366666666666667</v>
       </c>
     </row>
     <row r="8">
@@ -1459,16 +1459,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>it's pure vegetarian restaurant. all kind of item you would get. starting with breakfast pongal, rawa khichadi (upma), etc. veriety of dosa, every day there is one special dosa.. today it was paneer dosa... you also get dumplings , mini …</t>
+          <t>wide range of traditional indian sweets and savories. attending staff at sweet counter were very helpful. the staff went extra mile to pack the sweet boxes securely when she realized that i am bringing it back to my home country</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Service Quality</t>
+          <t>Cleanliness &amp; Restroom Hygiene</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.4850277232496833</v>
+        <v>0.3166666666666667</v>
       </c>
     </row>
     <row r="9">
@@ -1479,16 +1479,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>worst service got in lunch. i visited more than 40 a2bs around tamilnadu but this was very poor service. all servers are from other state and they don't know and understand tamil which cause so many chaos for my elders.</t>
+          <t>rating: 4 / 5 📍 key review points: 📌 location: …</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Service Quality</t>
+          <t>Food Variety &amp; Fast Service</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.3510511496918333</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10">
@@ -1499,16 +1499,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ordered poori and dosa from swiggy today. poori was dry and too oily. found a worm in chutney. i called to restaurant to inform this they didn’t answer me and hanged call.</t>
+          <t>had a great lunch at the restaurant. all the dishes tasted good. personally had the south indian meals. parking available maybe for 6-7 cars in the front, so a little congested during …</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Parking &amp; Accessibility</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.2602415752905459</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="11">
@@ -1519,16 +1519,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>worst ever service don't choose a2b shastri road better prefer shri sangeethas restaurant for quick dine service …</t>
+          <t>i visited the adyar ananda bhavan outlet in gandhipuram last night.the quantity and quality of the food were reasonably good, but the prices were on the higher side. however, the service style and the staff's demeanor were somewhat …</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Slow Service &amp; Staff Negligence</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.4680836175257094</v>
+        <v>0.4466666666666667</v>
       </c>
     </row>
     <row r="12">
@@ -1539,16 +1539,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>we stepped in during late hours for dinner. durga waited on us with a great smile. she managed to get all of the orders without making us wait for a longer time. i would definitely visit back especially to meet her again 🤪 …</t>
+          <t>lunch menu idli dosa, uttapam not available. dal, rice and vegetable menu served. taste and quality is good. staff is courteous.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Slow Service &amp; Staff Negligence</t>
+          <t>Food Variety &amp; Fast Service</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.4883630107730401</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="13">
@@ -1559,16 +1559,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>"i am writing to express my disappointment regarding the service at your restaurant during my recent visit. we waited for more than half an hour after being seated, but no staff member came to take our food order, even though we tried to …</t>
+          <t>it was an unplanned quick visit during our ride to kovai. just checked in to have some cool drinks, and the order process was tiring, and nobody was there to help with. got the order delivered only after 15 minutes that, too, just 2 orange …</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Slow Service &amp; Staff Negligence</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.331219954272798</v>
+        <v>0.4433333333333334</v>
       </c>
     </row>
     <row r="14">
@@ -1579,16 +1579,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>worst experience, around 30 mins, nobody came to table, they turned face other side. they never bother about customer. came out without having food, around 30 mins</t>
+          <t>hopeless! very rude staff. before boarding my bus, went in to get a coffee and take out breakfast. i was told to sit and someone would come and attend. waiters are just walking around . sat for 5 minutes. they keep talking to each other, but no one would attend. got frustrated and left. customer service is zero.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Slow Service &amp; Staff Negligence</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.4789770611466073</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="15">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>worst a2b restaurant i have ever seen no proper service persons . taking too long time to serve food . it should be closed or else change the manger or supervisor to take care</t>
+          <t>i had a sweet paniyaram which is very good taste but outer surface is very hard to bite which made my teeth painful. please make that as soft as possible to enjoy the delicious</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.4712951563330148</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="16">
@@ -1619,16 +1619,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>whatever you order its not there. dosa not there, manchurian not there …</t>
+          <t>we visited hotel and had to wait for a very long time. the servers were extremely slow and the service was delayed. this should not happen, especially for a place with such a good reputation. please ensure your staff attend to customers more quickly and efficiently.”</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.4914573385456499</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="17">
@@ -1639,67 +1639,67 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>very bad experience. it took 15 mins for someone to take the order. very few people are available for service. hardly any items are available, which is very surprising on a long weekend sunday. strictly not advisable for people planning to have a quick bite before boarding train.</t>
+          <t>limited options for jain food was available. jain food prepared was tasty. dodha burfi in sweets was too tasty. it just melts in mouth. i liked the sweets …</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Service Quality</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.4343627224523933</v>
+        <v>0.2733333333333333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Geetham</t>
+          <t>A2B</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>if you are looking for for south indian authentic vegetarian food. this is the place for you . don’t miss to taste paayasam that’s been served with every thali. quick service with happy meal</t>
+          <t>today during dinner, the service quality was very disappointing. none of the staff seemed attentive to customers. the waiters and captains were moving around without any focus, and there was no proper monitoring of the floor. …</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.4717969110226677</v>
+        <v>0.2933333333333333</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Geetham</t>
+          <t>A2B</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>quality of food degraded over the years. traditional tamilnadu meals quality is no more available in this resturant. high content of oil in every dish makes it unhealthy to eat at this place. resturant management should concentrate of food quality. service and atmosphere is decent and fast.</t>
+          <t>i have been visiting this place once in a while since 9 years. i just noticed that i never reviewed this place yet. the food here is exceptionally good usually though there was a small difference today. i would have reduced more stars for …</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Poor Experience &amp; Food Hygiene Complaints</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.4224800924759259</v>
+        <v>0.3433333333333333</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Geetham</t>
+          <t>A2B</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>nice ambience , clean restrooms , lovely food.. i love how they maintain their standards with consistency with respect to food.. loved their pista rose kunafa totally.. everything was delivered without delay, nice service.. overall a great experience! ♥️💐 …</t>
+          <t>visited on 10/09/2025 for breakfast. idli,wada, uttapa ordered. great taste.fast service.must drink coffee here.they have branches outside india also.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1708,27 +1708,27 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.4125097033794984</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Geetham</t>
+          <t>A2B</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>restaurant is very good, comforting and have very nice ambience. food is very good, all vegetarian menu and tastes very good. staff is also very nice, quite friendly and also able to understand hindi. menu is very vast including chinese, …</t>
+          <t>good for a vegetarian lunch and dinner. service is good with courteous staff. table cleaning is poor and so is the hand wash.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Food Variety &amp; Fast Service</t>
+          <t>Food Quantity &amp; Value for Money</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.4940951555090529</v>
+        <v>0.4533333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>